<commit_message>
Data: Update seed_data Excel from Jose's branch (Goldfields planillas, planning centers, pilots)
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seed_data/34_permits_to_work.xlsx
+++ b/seed_data/34_permits_to_work.xlsx
@@ -15029,10 +15029,8 @@
           <t>Trabajo eléctrico</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>500001</t>
-        </is>
+      <c r="C154" t="n">
+        <v>500001</v>
       </c>
       <c r="D154" t="inlineStr">
         <is>
@@ -15893,10 +15891,8 @@
           <t>Trabajo en altura</t>
         </is>
       </c>
-      <c r="C163" t="inlineStr">
-        <is>
-          <t>500001</t>
-        </is>
+      <c r="C163" t="n">
+        <v>500001</v>
       </c>
       <c r="D163" t="inlineStr">
         <is>

</xml_diff>